<commit_message>
feat: add gold upgrades and between-wave reinforcement choices
</commit_message>
<xml_diff>
--- a/configs/ElementGuardians_策划数值配置.xlsx
+++ b/configs/ElementGuardians_策划数值配置.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目概览" sheetId="1" r:id="Rf423633111cf47c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="防御塔" sheetId="2" r:id="R435cb8f5f9f548a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="敌人" sheetId="3" r:id="Re67106f68a354f92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="波次" sheetId="4" r:id="Rbb977f79452e46ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="强化" sheetId="5" r:id="R85277e1dbf7d4f8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经济参数" sheetId="6" r:id="Rbbc6bc054f4f4572"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全局参数" sheetId="7" r:id="R8a7fc49154624197"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值试算" sheetId="8" r:id="Rbacf7299071b4e6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目概览" sheetId="1" r:id="R514ed579b1eb4c35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="防御塔" sheetId="2" r:id="Rcc4827a319ab488b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="敌人" sheetId="3" r:id="Rbd45af0fd7f546b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="波次" sheetId="4" r:id="R0b3dddbd9b944376"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="强化" sheetId="5" r:id="R7e0c74d9637c4a1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经济参数" sheetId="6" r:id="Ra89a1d29e1fc4868"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全局参数" sheetId="7" r:id="Rf944a89df6fd4ff9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值试算" sheetId="8" r:id="R0cb42319a5144c47"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1312,6 +1312,28 @@
         <x:v>基地初始生命</x:v>
       </x:c>
     </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>tower_upgrade_lv2_cost</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>Lv1→Lv2费用，首版试验</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="12" t="str">
+        <x:v>tower_upgrade_lv3_cost</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
+        <x:v>Lv2→Lv3费用，首版试验</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>